<commit_message>
feat: herencia en Evento, cancelar operaciones en ventana y correcciones del feedback
- Evento pasa a ser clase padre de EventoEmergencia y EventoCapacitacion, cada una con sus reglas al asignar voluntarios
- Los getters de colecciones devuelven copias
- Fix: buscar/editar/eliminar un RUT con k minuscula y arrancar con un Excel vacio o dañado
- En modo ventana Cancelar vuelve al menu (OperacionCanceladaException)
- Menu de eventos con filtros por cupos y por prioridad, y menu de habilidades por voluntario
- Se quitan metodos duplicados o sin uso (getDisp, isDisponibilidad, mostrarHabilidades, mostrarVoluntarios, modificarVoluntario)
- Datos iniciales con un evento de cada tipo
</commit_message>
<xml_diff>
--- a/SGPV/sgpv_datos.xlsx
+++ b/SGPV/sgpv_datos.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="49">
   <si>
     <t>nombre</t>
   </si>
@@ -31,25 +31,37 @@
     <t>habilidades</t>
   </si>
   <si>
-    <t>Alfonso Perez</t>
-  </si>
-  <si>
-    <t>21034234-2</t>
+    <t>Juan Soto</t>
+  </si>
+  <si>
+    <t>22222222-2</t>
   </si>
   <si>
     <t>Quillota</t>
   </si>
   <si>
-    <t>Primeros Auxilios</t>
-  </si>
-  <si>
-    <t>Pepe Tapia</t>
-  </si>
-  <si>
-    <t>21049416-2</t>
-  </si>
-  <si>
-    <t>Cocinero</t>
+    <t>Primeros auxilios</t>
+  </si>
+  <si>
+    <t>Ana Pérez</t>
+  </si>
+  <si>
+    <t>11111111-1</t>
+  </si>
+  <si>
+    <t>Valparaíso</t>
+  </si>
+  <si>
+    <t>María Vidal</t>
+  </si>
+  <si>
+    <t>33333333-3</t>
+  </si>
+  <si>
+    <t>Con Con</t>
+  </si>
+  <si>
+    <t>Logística</t>
   </si>
   <si>
     <t>idPrograma</t>
@@ -82,46 +94,73 @@
     <t>rutsVoluntariosAsignados</t>
   </si>
   <si>
-    <t>P2</t>
-  </si>
-  <si>
-    <t>Emergencias</t>
-  </si>
-  <si>
-    <t>Bla bla bla</t>
-  </si>
-  <si>
-    <t>13-03-2026</t>
+    <t>tipo</t>
+  </si>
+  <si>
+    <t>habilidad</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>Reforestación Costera</t>
+  </si>
+  <si>
+    <t>Programa de plantación de árboles</t>
+  </si>
+  <si>
+    <t>01-03-2026</t>
+  </si>
+  <si>
+    <t>E1</t>
+  </si>
+  <si>
+    <t>Jornada de plantación</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>15-03-2026</t>
+  </si>
+  <si>
+    <t>NORMAL</t>
+  </si>
+  <si>
+    <t>REGULAR</t>
   </si>
   <si>
     <t>E2</t>
   </si>
   <si>
-    <t>Bla Blu Ble</t>
-  </si>
-  <si>
-    <t>Vinia del mar</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>30-03-2026</t>
-  </si>
-  <si>
-    <t>ALTA</t>
-  </si>
-  <si>
-    <t>P3</t>
-  </si>
-  <si>
-    <t>Prueba fecha</t>
-  </si>
-  <si>
-    <t>Fecha pa ver que pesque</t>
-  </si>
-  <si>
-    <t>21-04-2026</t>
+    <t>Respuesta a incendio forestal</t>
+  </si>
+  <si>
+    <t>20-03-2026</t>
+  </si>
+  <si>
+    <t>CATASTROFE</t>
+  </si>
+  <si>
+    <t>EMERGENCIA</t>
+  </si>
+  <si>
+    <t>E3</t>
+  </si>
+  <si>
+    <t>Curso de primeros auxilios</t>
+  </si>
+  <si>
+    <t>Sede central</t>
+  </si>
+  <si>
+    <t>25-03-2026</t>
+  </si>
+  <si>
+    <t>BAJA</t>
+  </si>
+  <si>
+    <t>CAPACITACION</t>
   </si>
 </sst>
 </file>
@@ -167,7 +206,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -198,7 +237,7 @@
         <v>7</v>
       </c>
       <c r="D2" t="b" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>8</v>
@@ -212,13 +251,30 @@
         <v>10</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D3" t="b" s="0">
         <v>1</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>11</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D4" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -228,49 +284,35 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>33</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>34</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -280,65 +322,147 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s" s="0">
         <v>0</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E1" t="s" s="0">
         <v>2</v>
       </c>
       <c r="F1" t="s" s="0">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G1" t="s" s="0">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="H1" t="s" s="0">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I1" t="s" s="0">
-        <v>21</v>
+        <v>25</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>27</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="G2" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="J2" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
         <v>28</v>
       </c>
-      <c r="E2" t="s" s="0">
-        <v>29</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>30</v>
-      </c>
-      <c r="G2" t="n" s="0">
-        <v>15.0</v>
-      </c>
-      <c r="H2" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="I2" t="s" s="0">
-        <v>6</v>
+      <c r="B3" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="G3" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="I3" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="J3" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="K3" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="G4" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="J4" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="K4" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>